<commit_message>
Updated files until today
</commit_message>
<xml_diff>
--- a/Grade3-Homeworks.xlsx
+++ b/Grade3-Homeworks.xlsx
@@ -17,12 +17,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>Monday</t>
-  </si>
-  <si>
-    <t>Date</t>
   </si>
   <si>
     <t xml:space="preserve">Telugu </t>
@@ -31,10 +28,10 @@
     <t xml:space="preserve">Maths </t>
   </si>
   <si>
-    <t>Tuesday</t>
+    <t>Date</t>
   </si>
   <si>
-    <t>Languages</t>
+    <t>Tuesday</t>
   </si>
   <si>
     <t xml:space="preserve">English </t>
@@ -43,13 +40,37 @@
     <t xml:space="preserve">Programming </t>
   </si>
   <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Languages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Science </t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Music</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Social </t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>KhatriHindiSanskrit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technology </t>
+  </si>
+  <si>
     <t>Telugu</t>
   </si>
   <si>
     <t>English</t>
-  </si>
-  <si>
-    <t>Wednesday</t>
   </si>
   <si>
     <t>Devanagari - HindiSanskritKhatriMarathi</t>
@@ -58,43 +79,22 @@
     <t>Maths</t>
   </si>
   <si>
-    <t xml:space="preserve">Science </t>
-  </si>
-  <si>
     <t>Technology</t>
   </si>
   <si>
     <t>Programming</t>
   </si>
   <si>
-    <t>Thursday</t>
-  </si>
-  <si>
-    <t>Music</t>
-  </si>
-  <si>
     <t>CarnaticMusic</t>
   </si>
   <si>
-    <t xml:space="preserve">Social </t>
-  </si>
-  <si>
     <t>Science</t>
-  </si>
-  <si>
-    <t>Friday</t>
   </si>
   <si>
     <t>SocialStudies ( + LifeSkills)</t>
   </si>
   <si>
     <t>Overview</t>
-  </si>
-  <si>
-    <t>KhatriHindiSanskrit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Technology </t>
   </si>
   <si>
     <t>HW: Complete 3rd class text book, work book, copy tracing book and get it verified by your parents</t>
@@ -130,6 +130,29 @@
   </si>
   <si>
     <t>HW: Make sure the website is updated with all the files for Grade 2 - All subjects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HW: Complete class 4 + class 5 AP Environment textbook + workboo
+</t>
+  </si>
+  <si>
+    <t>HW: Read the introduction again (Enlightened Education book - introduction)</t>
+  </si>
+  <si>
+    <t>HW: Complete class 4 + class 5 AP Environment textbook + workbook</t>
+  </si>
+  <si>
+    <t>HW: For 1 or 2 days, live without electricity;</t>
+  </si>
+  <si>
+    <t>HW: Play 'pillars' game
+Sthambhaala aata/Pillars game: Four players stand at and hold onto four different pillars, while a fifth player (the "thief" or IT) stands in the center. The four players try to quickly swap positions from one pillar to another without getting caught, while the central player tries to occupy an open pillar. Traditionally, it is a popular folk game played by children in rural Andhra Pradesh and Telangana, often during weddings under a marriage pandal (pelli pandiri).</t>
+  </si>
+  <si>
+    <t>HW: Read, write meanings, and answer exercises; Memorize all the sentences from the textbook. (Class 1 CBSE textbook)</t>
+  </si>
+  <si>
+    <t>HW: Practice these songs; Write down the raagam, thaalam, and swaras. (Practiced detecting swaras for songs - Keshava madhava; Animuthyaalandi sahajayoga songs)</t>
   </si>
 </sst>
 </file>
@@ -271,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -319,6 +342,9 @@
     </xf>
     <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,46 +563,48 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="3" max="12" width="19.38"/>
+    <col customWidth="1" min="3" max="10" width="19.38"/>
+    <col customWidth="1" min="11" max="11" width="22.88"/>
+    <col customWidth="1" min="12" max="12" width="21.88"/>
     <col hidden="1" min="13" max="23" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
@@ -844,7 +872,9 @@
       <c r="W11" s="7"/>
     </row>
     <row r="12">
-      <c r="A12" s="2"/>
+      <c r="A12" s="20">
+        <v>46296.0</v>
+      </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -853,8 +883,12 @@
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
+      <c r="J12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
@@ -869,18 +903,9 @@
       <c r="W12" s="7"/>
     </row>
     <row r="13">
-      <c r="A13" s="2"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
+      <c r="K13" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
@@ -894,18 +919,9 @@
       <c r="W13" s="7"/>
     </row>
     <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
+      <c r="K14" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
@@ -919,18 +935,9 @@
       <c r="W14" s="7"/>
     </row>
     <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
+      <c r="K15" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
@@ -944,15 +951,21 @@
       <c r="W15" s="7"/>
     </row>
     <row r="16">
-      <c r="A16" s="2"/>
+      <c r="A16" s="20">
+        <v>46297.0</v>
+      </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
+      <c r="E16" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
+      <c r="I16" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -25569,7 +25582,7 @@
       <c r="W1000" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="44">
     <mergeCell ref="I2:I4"/>
     <mergeCell ref="J2:J4"/>
     <mergeCell ref="K2:K4"/>
@@ -25581,12 +25594,10 @@
     <mergeCell ref="F2:F4"/>
     <mergeCell ref="G2:G4"/>
     <mergeCell ref="H2:H4"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="I5:I8"/>
+    <mergeCell ref="J5:J8"/>
+    <mergeCell ref="K5:K8"/>
+    <mergeCell ref="L5:L8"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="B5:B8"/>
     <mergeCell ref="C5:C8"/>
@@ -25594,15 +25605,28 @@
     <mergeCell ref="F5:F8"/>
     <mergeCell ref="G5:G8"/>
     <mergeCell ref="H5:H8"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
     <mergeCell ref="K10:K11"/>
     <mergeCell ref="L10:L11"/>
-    <mergeCell ref="I5:I8"/>
-    <mergeCell ref="J5:J8"/>
-    <mergeCell ref="K5:K8"/>
-    <mergeCell ref="L5:L8"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="I12:I15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="F12:F15"/>
+    <mergeCell ref="G12:G15"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
     <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -25621,10 +25645,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -25632,43 +25656,43 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1"/>

</xml_diff>